<commit_message>
Blue Wolf v0.0.8: vazifalar
- Vazifalar tabi subtablar bilan: Orqaga · Kundalik · Haftalik · Oylik
- Kundalik 4, haftalik 4, oylik 3 vazifa (har oʻyinchiga urugʻ bilan),
  davr sandiqlari, kun kombosi (×1.6 gacha), 7 kunlik kirish taqvimi
- Mukofot faqat resurs (qurilish resurslari + goʻsht), jami kuniga ≤ 37%
  kunlik ishlab chiqarish; balans tekshiruvi qoʻshildi
- Server: player_quests, QuestService, QuestFormula (= game.js),
  GET /quests, POST /quests/claim, /quests/login; harakatlar avtomatik sanaladi
- GDD bo'lim 14, Excel Sozlamalar, API va sxema yangilandi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014DHtibjv86AYXcpEPUVWXf
</commit_message>
<xml_diff>
--- a/docs/blue_wolf/blue_wolf_darajalar.xlsx
+++ b/docs/blue_wolf/blue_wolf_darajalar.xlsx
@@ -138,6 +138,7 @@
     <definedName function="false" hidden="false" name="hunt_mid_injury" vbProcedure="false">Sozlamalar!$B$321</definedName>
     <definedName function="false" hidden="false" name="hunt_small_party_penalty" vbProcedure="false">Sozlamalar!$B$260</definedName>
     <definedName function="false" hidden="false" name="hunt_speed_kmh" vbProcedure="false">Sozlamalar!$B$314</definedName>
+    <definedName function="false" hidden="false" name="login_gift_step" vbProcedure="false">Sozlamalar!$B$335</definedName>
     <definedName function="false" hidden="false" name="loot_cap_ratio" vbProcedure="false">Sozlamalar!$B$222</definedName>
     <definedName function="false" hidden="false" name="loot_carry_base" vbProcedure="false">Sozlamalar!$B$220</definedName>
     <definedName function="false" hidden="false" name="loot_carry_tier" vbProcedure="false">Sozlamalar!$B$221</definedName>
@@ -194,12 +195,21 @@
     <definedName function="false" hidden="false" name="promote_cost_share" vbProcedure="false">Sozlamalar!$B$46</definedName>
     <definedName function="false" hidden="false" name="promote_loss" vbProcedure="false">Sozlamalar!$B$45</definedName>
     <definedName function="false" hidden="false" name="promote_time_share" vbProcedure="false">Sozlamalar!$B$47</definedName>
+    <definedName function="false" hidden="false" name="quest_combo_max_days" vbProcedure="false">Sozlamalar!$B$332</definedName>
+    <definedName function="false" hidden="false" name="quest_combo_step" vbProcedure="false">Sozlamalar!$B$331</definedName>
     <definedName function="false" hidden="false" name="quest_daily_cap" vbProcedure="false">Sozlamalar!$B$36</definedName>
+    <definedName function="false" hidden="false" name="quest_daily_chest" vbProcedure="false">Sozlamalar!$B$330</definedName>
     <definedName function="false" hidden="false" name="quest_daily_count" vbProcedure="false">Sozlamalar!$B$34</definedName>
+    <definedName function="false" hidden="false" name="quest_meat_ratio" vbProcedure="false">Sozlamalar!$B$336</definedName>
     <definedName function="false" hidden="false" name="quest_milestone_cap" vbProcedure="false">Sozlamalar!$B$38</definedName>
+    <definedName function="false" hidden="false" name="quest_monthly_cap" vbProcedure="false">Sozlamalar!$B$329</definedName>
+    <definedName function="false" hidden="false" name="quest_monthly_chest" vbProcedure="false">Sozlamalar!$B$334</definedName>
+    <definedName function="false" hidden="false" name="quest_monthly_count" vbProcedure="false">Sozlamalar!$B$328</definedName>
     <definedName function="false" hidden="false" name="quest_safe_cap" vbProcedure="false">Sozlamalar!$B$40</definedName>
     <definedName function="false" hidden="false" name="quest_speedup_min" vbProcedure="false">Sozlamalar!$B$39</definedName>
+    <definedName function="false" hidden="false" name="quest_tz_offset_h" vbProcedure="false">Sozlamalar!$B$337</definedName>
     <definedName function="false" hidden="false" name="quest_weekly_cap" vbProcedure="false">Sozlamalar!$B$37</definedName>
+    <definedName function="false" hidden="false" name="quest_weekly_chest" vbProcedure="false">Sozlamalar!$B$333</definedName>
     <definedName function="false" hidden="false" name="quest_weekly_count" vbProcedure="false">Sozlamalar!$B$35</definedName>
     <definedName function="false" hidden="false" name="queue_cancel_refund" vbProcedure="false">Sozlamalar!$B$301</definedName>
     <definedName function="false" hidden="false" name="raid_coef" vbProcedure="false">Sozlamalar!$B$223</definedName>
@@ -328,7 +338,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2679" uniqueCount="1948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2710" uniqueCount="1970">
   <si>
     <t xml:space="preserve">Blue Wolf — oʻyinchi darajalari (1–25)</t>
   </si>
@@ -6163,6 +6173,72 @@
   </si>
   <si>
     <t xml:space="preserve">… + tasodifiy 0–shu (kartaga qarab)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vazifalar: oylik va mukofotlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oylik vazifa soni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Har oy (kalendar oy) 3 ta vazifa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oylik mukofot chegarasi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oylik vazifalar jami = kunlik ishlab chiqarish × shu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kun kombosi sandigʻi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kunning hamma vazifasi bajarilganda (× kombo koeff.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kombo qadami</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ulush/kun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ketma-ket har kun uchun sandiq +shu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kombo maksimal kuni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shundan keyin oʻsmaydi (maks ×1.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haftalik sandiq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haftaning hamma vazifasi bajarilganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oylik sandiq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oyning hamma vazifasi bajarilganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kirish sovgʻasi qadami</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 kunlik taqvim: n-kun = shu × n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vazifa goʻshti koeffitsienti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goʻsht mukofoti = ulush × shu × toʻdaning kunlik goʻsht ehtiyoji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vazifalar vaqt mintaqasi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kun/hafta/oy chegarasi: UTC+shu (Toshkent)</t>
   </si>
   <si>
     <t xml:space="preserve">Izoh: vazn ustuni haqiqiy zoologik maʼlumotlarga (oʻrtacha katta erkak boʻri vazni) asoslangan; mifologik boʻrilarda vazn yoʻq.</t>
@@ -22687,7 +22763,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A3:D330"/>
+  <dimension ref="A3:D341"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
@@ -26734,7 +26810,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A316" s="2" t="s">
         <v>1925</v>
       </c>
@@ -26748,7 +26824,7 @@
         <v>1926</v>
       </c>
     </row>
-    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A317" s="2" t="s">
         <v>1927</v>
       </c>
@@ -26762,7 +26838,7 @@
         <v>1928</v>
       </c>
     </row>
-    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A318" s="2" t="s">
         <v>1929</v>
       </c>
@@ -26776,7 +26852,7 @@
         <v>1930</v>
       </c>
     </row>
-    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A319" s="2" t="s">
         <v>1931</v>
       </c>
@@ -26790,7 +26866,7 @@
         <v>1932</v>
       </c>
     </row>
-    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A320" s="2" t="s">
         <v>1933</v>
       </c>
@@ -26804,7 +26880,7 @@
         <v>1934</v>
       </c>
     </row>
-    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A321" s="2" t="s">
         <v>1935</v>
       </c>
@@ -26818,7 +26894,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A322" s="2" t="s">
         <v>1938</v>
       </c>
@@ -26832,7 +26908,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A323" s="2" t="s">
         <v>1939</v>
       </c>
@@ -26846,7 +26922,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A324" s="2" t="s">
         <v>1940</v>
       </c>
@@ -26860,7 +26936,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A325" s="2" t="s">
         <v>1941</v>
       </c>
@@ -26874,7 +26950,7 @@
         <v>1942</v>
       </c>
     </row>
-    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A326" s="2" t="s">
         <v>1943</v>
       </c>
@@ -26888,19 +26964,164 @@
         <v>1944</v>
       </c>
     </row>
-    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A327" s="2" t="s">
+        <v>1945</v>
+      </c>
+    </row>
+    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A328" s="2" t="s">
-        <v>1945</v>
-      </c>
-    </row>
-    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1946</v>
+      </c>
+      <c r="B328" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C328" s="2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D328" s="2" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A329" s="2" t="s">
-        <v>1946</v>
-      </c>
-    </row>
-    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1948</v>
+      </c>
+      <c r="B329" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C329" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D329" s="2" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A330" s="2" t="s">
-        <v>1947</v>
+        <v>1950</v>
+      </c>
+      <c r="B330" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C330" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D330" s="2" t="s">
+        <v>1951</v>
+      </c>
+    </row>
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A331" s="2" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B331" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C331" s="2" t="s">
+        <v>1953</v>
+      </c>
+      <c r="D331" s="2" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A332" s="2" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B332" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C332" s="2" t="s">
+        <v>1455</v>
+      </c>
+      <c r="D332" s="2" t="s">
+        <v>1956</v>
+      </c>
+    </row>
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A333" s="2" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B333" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C333" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D333" s="2" t="s">
+        <v>1958</v>
+      </c>
+    </row>
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A334" s="2" t="s">
+        <v>1959</v>
+      </c>
+      <c r="B334" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C334" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D334" s="2" t="s">
+        <v>1960</v>
+      </c>
+    </row>
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A335" s="2" t="s">
+        <v>1961</v>
+      </c>
+      <c r="B335" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C335" s="2" t="s">
+        <v>1953</v>
+      </c>
+      <c r="D335" s="2" t="s">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A336" s="2" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B336" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C336" s="2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="D336" s="2" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="2" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B337" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C337" s="2" t="s">
+        <v>1461</v>
+      </c>
+      <c r="D337" s="2" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="1" t="s">
+        <v>1967</v>
+      </c>
+    </row>
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="1" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="1" t="s">
+        <v>1969</v>
       </c>
     </row>
   </sheetData>

</xml_diff>